<commit_message>
Tabel Academic calendar aangepast. Weekenden voor en na de vakantie vallen onder de vakantie. Het weekend voor een tentamenperiode valt onder de tentamenperiode. Het weekend erna niet. Feestdagen tijdens tentamenperiodes vallen onder de tentamenperiode.
</commit_message>
<xml_diff>
--- a/Academic calendar.xlsx
+++ b/Academic calendar.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30120"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30125"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\betti\Documents\Hanze\Data mining\Assignment - ACLO (1)\Data (6)\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4D2162D-9618-430F-8F69-3C3BEA127384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAB2BA75-9429-4400-959D-10682590E3DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-9540" windowWidth="38640" windowHeight="21120" xr2:uid="{ECC1C42F-9541-4405-9BC9-4DA3EA29DB42}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1138" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1200" uniqueCount="6">
   <si>
     <t>Datum</t>
   </si>
@@ -1076,6 +1076,9 @@
       <c r="A90" s="1">
         <v>43036</v>
       </c>
+      <c r="D90" t="s">
+        <v>4</v>
+      </c>
       <c r="E90" t="s">
         <v>4</v>
       </c>
@@ -1084,6 +1087,9 @@
       <c r="A91" s="1">
         <v>43037</v>
       </c>
+      <c r="D91" t="s">
+        <v>4</v>
+      </c>
       <c r="E91" t="s">
         <v>4</v>
       </c>
@@ -1440,6 +1446,9 @@
       <c r="A146" s="1">
         <v>43092</v>
       </c>
+      <c r="C146" t="s">
+        <v>4</v>
+      </c>
       <c r="E146" t="s">
         <v>4</v>
       </c>
@@ -1448,6 +1457,9 @@
       <c r="A147" s="1">
         <v>43093</v>
       </c>
+      <c r="C147" t="s">
+        <v>4</v>
+      </c>
       <c r="E147" t="s">
         <v>4</v>
       </c>
@@ -1567,6 +1579,9 @@
       <c r="A160" s="1">
         <v>43106</v>
       </c>
+      <c r="C160" t="s">
+        <v>4</v>
+      </c>
       <c r="E160" t="s">
         <v>4</v>
       </c>
@@ -1575,6 +1590,9 @@
       <c r="A161" s="1">
         <v>43107</v>
       </c>
+      <c r="C161" t="s">
+        <v>4</v>
+      </c>
       <c r="E161" t="s">
         <v>4</v>
       </c>
@@ -1608,6 +1626,9 @@
       <c r="A167" s="1">
         <v>43113</v>
       </c>
+      <c r="D167" t="s">
+        <v>4</v>
+      </c>
       <c r="E167" t="s">
         <v>4</v>
       </c>
@@ -1616,6 +1637,9 @@
       <c r="A168" s="1">
         <v>43114</v>
       </c>
+      <c r="D168" t="s">
+        <v>4</v>
+      </c>
       <c r="E168" t="s">
         <v>4</v>
       </c>
@@ -2075,6 +2099,9 @@
       <c r="A237" s="1">
         <v>43183</v>
       </c>
+      <c r="D237" t="s">
+        <v>4</v>
+      </c>
       <c r="E237" t="s">
         <v>4</v>
       </c>
@@ -2083,6 +2110,9 @@
       <c r="A238" s="1">
         <v>43184</v>
       </c>
+      <c r="D238" t="s">
+        <v>4</v>
+      </c>
       <c r="E238" t="s">
         <v>4</v>
       </c>
@@ -2607,6 +2637,9 @@
       <c r="A314" s="1">
         <v>43260</v>
       </c>
+      <c r="D314" t="s">
+        <v>4</v>
+      </c>
       <c r="E314" t="s">
         <v>4</v>
       </c>
@@ -2615,6 +2648,9 @@
       <c r="A315" s="1">
         <v>43261</v>
       </c>
+      <c r="D315" t="s">
+        <v>4</v>
+      </c>
       <c r="E315" t="s">
         <v>4</v>
       </c>
@@ -3679,6 +3715,9 @@
       <c r="A454" s="1">
         <v>43400</v>
       </c>
+      <c r="D454" t="s">
+        <v>4</v>
+      </c>
       <c r="E454" t="s">
         <v>4</v>
       </c>
@@ -3687,6 +3726,9 @@
       <c r="A455" s="1">
         <v>43401</v>
       </c>
+      <c r="D455" t="s">
+        <v>4</v>
+      </c>
       <c r="E455" t="s">
         <v>4</v>
       </c>
@@ -4043,6 +4085,9 @@
       <c r="A510" s="1">
         <v>43456</v>
       </c>
+      <c r="C510" t="s">
+        <v>4</v>
+      </c>
       <c r="E510" t="s">
         <v>4</v>
       </c>
@@ -4051,6 +4096,9 @@
       <c r="A511" s="1">
         <v>43457</v>
       </c>
+      <c r="C511" t="s">
+        <v>4</v>
+      </c>
       <c r="E511" t="s">
         <v>4</v>
       </c>
@@ -4170,6 +4218,9 @@
       <c r="A524" s="1">
         <v>43470</v>
       </c>
+      <c r="C524" t="s">
+        <v>4</v>
+      </c>
       <c r="E524" t="s">
         <v>4</v>
       </c>
@@ -4178,6 +4229,9 @@
       <c r="A525" s="1">
         <v>43471</v>
       </c>
+      <c r="C525" t="s">
+        <v>4</v>
+      </c>
       <c r="E525" t="s">
         <v>4</v>
       </c>
@@ -4211,6 +4265,9 @@
       <c r="A531" s="1">
         <v>43477</v>
       </c>
+      <c r="D531" t="s">
+        <v>4</v>
+      </c>
       <c r="E531" t="s">
         <v>4</v>
       </c>
@@ -4219,6 +4276,9 @@
       <c r="A532" s="1">
         <v>43478</v>
       </c>
+      <c r="D532" t="s">
+        <v>4</v>
+      </c>
       <c r="E532" t="s">
         <v>4</v>
       </c>
@@ -4678,6 +4738,9 @@
       <c r="A601" s="1">
         <v>43547</v>
       </c>
+      <c r="D601" t="s">
+        <v>4</v>
+      </c>
       <c r="E601" t="s">
         <v>4</v>
       </c>
@@ -4686,6 +4749,9 @@
       <c r="A602" s="1">
         <v>43548</v>
       </c>
+      <c r="D602" t="s">
+        <v>4</v>
+      </c>
       <c r="E602" t="s">
         <v>4</v>
       </c>
@@ -5212,6 +5278,9 @@
       <c r="A679" s="1">
         <v>43625</v>
       </c>
+      <c r="D679" t="s">
+        <v>4</v>
+      </c>
       <c r="E679" t="s">
         <v>4</v>
       </c>
@@ -5223,6 +5292,9 @@
       <c r="B680" t="s">
         <v>4</v>
       </c>
+      <c r="D680" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="681" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A681" s="1">
@@ -5384,6 +5456,9 @@
       <c r="A699" s="1">
         <v>43645</v>
       </c>
+      <c r="C699" t="s">
+        <v>4</v>
+      </c>
       <c r="E699" t="s">
         <v>4</v>
       </c>
@@ -5392,6 +5467,9 @@
       <c r="A700" s="1">
         <v>43646</v>
       </c>
+      <c r="C700" t="s">
+        <v>4</v>
+      </c>
       <c r="E700" t="s">
         <v>4</v>
       </c>
@@ -6273,6 +6351,9 @@
       <c r="A818" s="1">
         <v>43764</v>
       </c>
+      <c r="D818" t="s">
+        <v>4</v>
+      </c>
       <c r="E818" t="s">
         <v>4</v>
       </c>
@@ -6281,6 +6362,9 @@
       <c r="A819" s="1">
         <v>43765</v>
       </c>
+      <c r="D819" t="s">
+        <v>4</v>
+      </c>
       <c r="E819" t="s">
         <v>4</v>
       </c>
@@ -6637,6 +6721,9 @@
       <c r="A874" s="1">
         <v>43820</v>
       </c>
+      <c r="C874" t="s">
+        <v>4</v>
+      </c>
       <c r="E874" t="s">
         <v>4</v>
       </c>
@@ -6645,6 +6732,9 @@
       <c r="A875" s="1">
         <v>43821</v>
       </c>
+      <c r="C875" t="s">
+        <v>4</v>
+      </c>
       <c r="E875" t="s">
         <v>4</v>
       </c>
@@ -6764,6 +6854,9 @@
       <c r="A888" s="1">
         <v>43834</v>
       </c>
+      <c r="C888" t="s">
+        <v>4</v>
+      </c>
       <c r="E888" t="s">
         <v>4</v>
       </c>
@@ -6772,6 +6865,9 @@
       <c r="A889" s="1">
         <v>43835</v>
       </c>
+      <c r="C889" t="s">
+        <v>4</v>
+      </c>
       <c r="E889" t="s">
         <v>4</v>
       </c>
@@ -6805,6 +6901,9 @@
       <c r="A895" s="1">
         <v>43841</v>
       </c>
+      <c r="D895" t="s">
+        <v>4</v>
+      </c>
       <c r="E895" t="s">
         <v>4</v>
       </c>
@@ -6813,6 +6912,9 @@
       <c r="A896" s="1">
         <v>43842</v>
       </c>
+      <c r="D896" t="s">
+        <v>4</v>
+      </c>
       <c r="E896" t="s">
         <v>4</v>
       </c>
@@ -7272,6 +7374,9 @@
       <c r="A965" s="1">
         <v>43911</v>
       </c>
+      <c r="D965" t="s">
+        <v>4</v>
+      </c>
       <c r="E965" t="s">
         <v>4</v>
       </c>
@@ -7280,6 +7385,9 @@
       <c r="A966" s="1">
         <v>43912</v>
       </c>
+      <c r="D966" t="s">
+        <v>4</v>
+      </c>
       <c r="E966" t="s">
         <v>4</v>
       </c>
@@ -7801,6 +7909,9 @@
       <c r="A1042" s="1">
         <v>43988</v>
       </c>
+      <c r="D1042" t="s">
+        <v>4</v>
+      </c>
       <c r="E1042" t="s">
         <v>4</v>
       </c>
@@ -7809,6 +7920,9 @@
       <c r="A1043" s="1">
         <v>43989</v>
       </c>
+      <c r="D1043" t="s">
+        <v>4</v>
+      </c>
       <c r="E1043" t="s">
         <v>4</v>
       </c>
@@ -8105,6 +8219,9 @@
       <c r="A1077" s="1">
         <v>44023</v>
       </c>
+      <c r="C1077" t="s">
+        <v>4</v>
+      </c>
       <c r="E1077" t="s">
         <v>4</v>
       </c>
@@ -8113,6 +8230,9 @@
       <c r="A1078" s="1">
         <v>44024</v>
       </c>
+      <c r="C1078" t="s">
+        <v>4</v>
+      </c>
       <c r="E1078" t="s">
         <v>4</v>
       </c>
@@ -8412,6 +8532,9 @@
       <c r="C1112" t="s">
         <v>4</v>
       </c>
+      <c r="D1112" t="s">
+        <v>4</v>
+      </c>
       <c r="E1112" t="s">
         <v>4</v>
       </c>
@@ -8423,6 +8546,9 @@
       <c r="C1113" t="s">
         <v>4</v>
       </c>
+      <c r="D1113" t="s">
+        <v>4</v>
+      </c>
       <c r="E1113" t="s">
         <v>4</v>
       </c>
@@ -8903,6 +9029,9 @@
       <c r="A1182" s="1">
         <v>44128</v>
       </c>
+      <c r="D1182" t="s">
+        <v>4</v>
+      </c>
       <c r="E1182" t="s">
         <v>4</v>
       </c>
@@ -8911,6 +9040,9 @@
       <c r="A1183" s="1">
         <v>44129</v>
       </c>
+      <c r="D1183" t="s">
+        <v>4</v>
+      </c>
       <c r="E1183" t="s">
         <v>4</v>
       </c>
@@ -9267,6 +9399,9 @@
       <c r="A1238" s="1">
         <v>44184</v>
       </c>
+      <c r="C1238" t="s">
+        <v>4</v>
+      </c>
       <c r="E1238" t="s">
         <v>4</v>
       </c>
@@ -9275,6 +9410,9 @@
       <c r="A1239" s="1">
         <v>44185</v>
       </c>
+      <c r="C1239" t="s">
+        <v>4</v>
+      </c>
       <c r="E1239" t="s">
         <v>4</v>
       </c>
@@ -9394,6 +9532,9 @@
       <c r="A1252" s="1">
         <v>44198</v>
       </c>
+      <c r="C1252" t="s">
+        <v>4</v>
+      </c>
       <c r="E1252" t="s">
         <v>4</v>
       </c>
@@ -9402,6 +9543,9 @@
       <c r="A1253" s="1">
         <v>44199</v>
       </c>
+      <c r="C1253" t="s">
+        <v>4</v>
+      </c>
       <c r="E1253" t="s">
         <v>4</v>
       </c>
@@ -9435,6 +9579,9 @@
       <c r="A1259" s="1">
         <v>44205</v>
       </c>
+      <c r="D1259" t="s">
+        <v>4</v>
+      </c>
       <c r="E1259" t="s">
         <v>4</v>
       </c>
@@ -9443,6 +9590,9 @@
       <c r="A1260" s="1">
         <v>44206</v>
       </c>
+      <c r="D1260" t="s">
+        <v>4</v>
+      </c>
       <c r="E1260" t="s">
         <v>4</v>
       </c>
@@ -9902,6 +10052,9 @@
       <c r="A1329" s="1">
         <v>44275</v>
       </c>
+      <c r="D1329" t="s">
+        <v>4</v>
+      </c>
       <c r="E1329" t="s">
         <v>4</v>
       </c>
@@ -9910,6 +10063,9 @@
       <c r="A1330" s="1">
         <v>44276</v>
       </c>
+      <c r="D1330" t="s">
+        <v>4</v>
+      </c>
       <c r="E1330" t="s">
         <v>4</v>
       </c>
@@ -10015,11 +10171,17 @@
       <c r="B1342" t="s">
         <v>4</v>
       </c>
+      <c r="D1342" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="1343" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1343" s="1">
         <v>44289</v>
       </c>
+      <c r="D1343" t="s">
+        <v>4</v>
+      </c>
       <c r="E1343" t="s">
         <v>4</v>
       </c>
@@ -10031,6 +10193,9 @@
       <c r="B1344" t="s">
         <v>4</v>
       </c>
+      <c r="D1344" t="s">
+        <v>4</v>
+      </c>
       <c r="E1344" t="s">
         <v>4</v>
       </c>
@@ -10042,6 +10207,9 @@
       <c r="B1345" t="s">
         <v>4</v>
       </c>
+      <c r="D1345" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="1346" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1346" s="1">
@@ -10422,6 +10590,9 @@
       <c r="A1406" s="1">
         <v>44352</v>
       </c>
+      <c r="D1406" t="s">
+        <v>4</v>
+      </c>
       <c r="E1406" t="s">
         <v>4</v>
       </c>
@@ -10430,6 +10601,9 @@
       <c r="A1407" s="1">
         <v>44353</v>
       </c>
+      <c r="D1407" t="s">
+        <v>4</v>
+      </c>
       <c r="E1407" t="s">
         <v>4</v>
       </c>
@@ -10726,6 +10900,9 @@
       <c r="A1441" s="1">
         <v>44387</v>
       </c>
+      <c r="C1441" t="s">
+        <v>4</v>
+      </c>
       <c r="E1441" t="s">
         <v>4</v>
       </c>
@@ -10734,6 +10911,9 @@
       <c r="A1442" s="1">
         <v>44388</v>
       </c>
+      <c r="C1442" t="s">
+        <v>4</v>
+      </c>
       <c r="E1442" t="s">
         <v>4</v>
       </c>
@@ -11550,6 +11730,9 @@
       <c r="A1553" s="1">
         <v>44499</v>
       </c>
+      <c r="D1553" t="s">
+        <v>4</v>
+      </c>
       <c r="E1553" t="s">
         <v>4</v>
       </c>
@@ -11557,6 +11740,9 @@
     <row r="1554" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1554" s="1">
         <v>44500</v>
+      </c>
+      <c r="D1554" t="s">
+        <v>4</v>
       </c>
       <c r="E1554" t="s">
         <v>4</v>

</xml_diff>